<commit_message>
- Updated translations - Code cleaning - Reports templates cleaning
</commit_message>
<xml_diff>
--- a/api/templates/xpert_test_activities_report/en.xlsx
+++ b/api/templates/xpert_test_activities_report/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\xpert_test_activities_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D212C8A3-8439-419F-B0C8-C8239610977F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F590DD-7817-478B-92B3-4A04B17DEB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{ECDE60A4-9CFB-4908-8281-3FECAA6944A5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ECDE60A4-9CFB-4908-8281-3FECAA6944A5}"/>
   </bookViews>
   <sheets>
     <sheet name="M4B2.Activities report" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <r>
       <t xml:space="preserve">                            MINISTRY OF HEALTH                                                                                                         </t>
@@ -167,10 +167,22 @@
     <t xml:space="preserve">Email: </t>
   </si>
   <si>
-    <t xml:space="preserve">Date Range:      </t>
-  </si>
-  <si>
     <t>Other errors</t>
+  </si>
+  <si>
+    <t>&lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserFullName&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserMobilePhone&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserEmail&gt;</t>
   </si>
 </sst>
 </file>
@@ -420,10 +432,6 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -467,6 +475,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -820,43 +832,47 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="20.25">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-    </row>
-    <row r="5" spans="1:9" ht="17.25">
-      <c r="A5" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+    </row>
+    <row r="5" spans="1:9" ht="17.25" customHeight="1">
+      <c r="A5" s="38" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
     </row>
     <row r="6" spans="1:9" ht="16.5">
       <c r="A6" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
+      <c r="B6" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
     </row>
     <row r="7" spans="1:9" ht="16.5">
       <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="5"/>
+      <c r="B7" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="C7" s="5"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -866,223 +882,227 @@
       <c r="A8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="D8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
       <c r="F9" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="16.5">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
       <c r="F10" s="7">
         <f>F11+F12+F13+F14+F15+F16</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="16.5">
-      <c r="A11" s="31"/>
-      <c r="B11" s="32" t="s">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:9" ht="16.5">
-      <c r="A12" s="31"/>
-      <c r="B12" s="32" t="s">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:9" ht="16.5">
-      <c r="A13" s="31"/>
-      <c r="B13" s="32" t="s">
+      <c r="A13" s="30"/>
+      <c r="B13" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:9" ht="16.5">
-      <c r="A14" s="31"/>
-      <c r="B14" s="28" t="s">
+      <c r="A14" s="30"/>
+      <c r="B14" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:9" ht="16.5">
-      <c r="A15" s="31"/>
-      <c r="B15" s="28" t="s">
+      <c r="A15" s="30"/>
+      <c r="B15" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:9" ht="16.5">
-      <c r="A16" s="37"/>
-      <c r="B16" s="29" t="s">
+      <c r="A16" s="36"/>
+      <c r="B16" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
       <c r="F16" s="9">
         <f>SUM(F17:F28)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16.5">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="16.5">
-      <c r="A18" s="31"/>
-      <c r="B18" s="32" t="s">
+      <c r="A18" s="30"/>
+      <c r="B18" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
       <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="16.5">
-      <c r="A19" s="31"/>
-      <c r="B19" s="32" t="s">
+      <c r="A19" s="30"/>
+      <c r="B19" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="16.5">
-      <c r="A20" s="31"/>
-      <c r="B20" s="32" t="s">
+      <c r="A20" s="30"/>
+      <c r="B20" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="16.5">
-      <c r="A21" s="31"/>
-      <c r="B21" s="32" t="s">
+      <c r="A21" s="30"/>
+      <c r="B21" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6" ht="16.5">
-      <c r="A22" s="31"/>
-      <c r="B22" s="32" t="s">
+      <c r="A22" s="30"/>
+      <c r="B22" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" ht="16.5">
-      <c r="A23" s="31"/>
-      <c r="B23" s="32" t="s">
+      <c r="A23" s="30"/>
+      <c r="B23" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
       <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6" ht="16.5">
-      <c r="A24" s="31"/>
-      <c r="B24" s="32" t="s">
+      <c r="A24" s="30"/>
+      <c r="B24" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:6" ht="16.5">
-      <c r="A25" s="31"/>
-      <c r="B25" s="32" t="s">
+      <c r="A25" s="30"/>
+      <c r="B25" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="31"/>
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:6" ht="16.5">
-      <c r="A26" s="31"/>
-      <c r="B26" s="32" t="s">
+      <c r="A26" s="30"/>
+      <c r="B26" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6" ht="16.5">
-      <c r="A27" s="31"/>
-      <c r="B27" s="32" t="s">
+      <c r="A27" s="30"/>
+      <c r="B27" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6" ht="16.5">
-      <c r="A28" s="31"/>
-      <c r="B28" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
+      <c r="A28" s="30"/>
+      <c r="B28" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
       <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6" ht="16.5">
@@ -1148,39 +1168,39 @@
     <row r="35" spans="1:6" ht="16.5">
       <c r="A35" s="20"/>
       <c r="B35" s="20"/>
-      <c r="C35" s="26" t="s">
+      <c r="C35" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
     </row>
     <row r="36" spans="1:6" ht="16.5">
       <c r="A36" s="21" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="22"/>
-      <c r="C36" s="27" t="s">
+      <c r="C36" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D36" s="27"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="27"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
     </row>
     <row r="37" spans="1:6" ht="16.5">
       <c r="A37" s="23" t="s">
         <v>36</v>
       </c>
       <c r="B37" s="23"/>
-      <c r="C37" s="26" t="s">
+      <c r="C37" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A10:A16"/>
@@ -1190,6 +1210,7 @@
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B6:I6"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A17:A28"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B18:E18"/>

</xml_diff>